<commit_message>
[feat] 44 - LootingUI Finished
- LootingUI 제작 완료
- 추후 폰트 및 효과 수정치 적용 필요
</commit_message>
<xml_diff>
--- a/Assets/Resources/CSVData/levelEXP.xlsx
+++ b/Assets/Resources/CSVData/levelEXP.xlsx
@@ -353,602 +353,602 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1">
-        <f t="shared" ref="A1:A6" si="0">ROW(A1) * 100</f>
-        <v>100</v>
+        <f>ROW(A1) * 2 + 3</f>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2">
-        <f t="shared" si="0"/>
-        <v>200</v>
+        <f t="shared" ref="A2:A65" si="0">ROW(A2) * 2 + 3</f>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>500</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>600</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7">
-        <f>ROW(A7) * 100</f>
-        <v>700</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8">
-        <f t="shared" ref="A8:A71" si="1">ROW(A8) * 100</f>
-        <v>800</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9">
-        <f t="shared" si="1"/>
-        <v>900</v>
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10">
-        <f t="shared" si="1"/>
-        <v>1000</v>
+        <f t="shared" si="0"/>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11">
-        <f t="shared" si="1"/>
-        <v>1100</v>
+        <f t="shared" si="0"/>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12">
-        <f t="shared" si="1"/>
-        <v>1200</v>
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13">
-        <f t="shared" si="1"/>
-        <v>1300</v>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14">
-        <f t="shared" si="1"/>
-        <v>1400</v>
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15">
-        <f t="shared" si="1"/>
-        <v>1500</v>
+        <f t="shared" si="0"/>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16">
-        <f t="shared" si="1"/>
-        <v>1600</v>
+        <f t="shared" si="0"/>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17">
-        <f t="shared" si="1"/>
-        <v>1700</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18">
-        <f t="shared" si="1"/>
-        <v>1800</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19">
-        <f t="shared" si="1"/>
-        <v>1900</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20">
-        <f t="shared" si="1"/>
-        <v>2000</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21">
-        <f t="shared" si="1"/>
-        <v>2100</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22">
-        <f t="shared" si="1"/>
-        <v>2200</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23">
-        <f t="shared" si="1"/>
-        <v>2300</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24">
-        <f t="shared" si="1"/>
-        <v>2400</v>
+        <f t="shared" si="0"/>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25">
-        <f t="shared" si="1"/>
-        <v>2500</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26">
-        <f t="shared" si="1"/>
-        <v>2600</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27">
-        <f t="shared" si="1"/>
-        <v>2700</v>
+        <f t="shared" si="0"/>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28">
-        <f t="shared" si="1"/>
-        <v>2800</v>
+        <f t="shared" si="0"/>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29">
-        <f t="shared" si="1"/>
-        <v>2900</v>
+        <f t="shared" si="0"/>
+        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30">
-        <f t="shared" si="1"/>
-        <v>3000</v>
+        <f t="shared" si="0"/>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31">
-        <f t="shared" si="1"/>
-        <v>3100</v>
+        <f t="shared" si="0"/>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32">
-        <f t="shared" si="1"/>
-        <v>3200</v>
+        <f t="shared" si="0"/>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33">
-        <f t="shared" si="1"/>
-        <v>3300</v>
+        <f t="shared" si="0"/>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34">
-        <f t="shared" si="1"/>
-        <v>3400</v>
+        <f t="shared" si="0"/>
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35">
-        <f t="shared" si="1"/>
-        <v>3500</v>
+        <f t="shared" si="0"/>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36">
-        <f t="shared" si="1"/>
-        <v>3600</v>
+        <f t="shared" si="0"/>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37">
-        <f t="shared" si="1"/>
-        <v>3700</v>
+        <f t="shared" si="0"/>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38">
-        <f t="shared" si="1"/>
-        <v>3800</v>
+        <f t="shared" si="0"/>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39">
-        <f t="shared" si="1"/>
-        <v>3900</v>
+        <f t="shared" si="0"/>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40">
-        <f t="shared" si="1"/>
-        <v>4000</v>
+        <f t="shared" si="0"/>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41">
-        <f t="shared" si="1"/>
-        <v>4100</v>
+        <f t="shared" si="0"/>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42">
-        <f t="shared" si="1"/>
-        <v>4200</v>
+        <f t="shared" si="0"/>
+        <v>87</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43">
-        <f t="shared" si="1"/>
-        <v>4300</v>
+        <f t="shared" si="0"/>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44">
-        <f t="shared" si="1"/>
-        <v>4400</v>
+        <f t="shared" si="0"/>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45">
-        <f t="shared" si="1"/>
-        <v>4500</v>
+        <f t="shared" si="0"/>
+        <v>93</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46">
-        <f t="shared" si="1"/>
-        <v>4600</v>
+        <f t="shared" si="0"/>
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47">
-        <f t="shared" si="1"/>
-        <v>4700</v>
+        <f t="shared" si="0"/>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48">
-        <f t="shared" si="1"/>
-        <v>4800</v>
+        <f t="shared" si="0"/>
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49">
-        <f t="shared" si="1"/>
-        <v>4900</v>
+        <f t="shared" si="0"/>
+        <v>101</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50">
-        <f t="shared" si="1"/>
-        <v>5000</v>
+        <f t="shared" si="0"/>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51">
-        <f t="shared" si="1"/>
-        <v>5100</v>
+        <f t="shared" si="0"/>
+        <v>105</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52">
-        <f t="shared" si="1"/>
-        <v>5200</v>
+        <f t="shared" si="0"/>
+        <v>107</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53">
-        <f t="shared" si="1"/>
-        <v>5300</v>
+        <f t="shared" si="0"/>
+        <v>109</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54">
-        <f t="shared" si="1"/>
-        <v>5400</v>
+        <f t="shared" si="0"/>
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55">
-        <f t="shared" si="1"/>
-        <v>5500</v>
+        <f t="shared" si="0"/>
+        <v>113</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56">
-        <f t="shared" si="1"/>
-        <v>5600</v>
+        <f t="shared" si="0"/>
+        <v>115</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57">
-        <f t="shared" si="1"/>
-        <v>5700</v>
+        <f t="shared" si="0"/>
+        <v>117</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58">
-        <f t="shared" si="1"/>
-        <v>5800</v>
+        <f t="shared" si="0"/>
+        <v>119</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59">
-        <f t="shared" si="1"/>
-        <v>5900</v>
+        <f t="shared" si="0"/>
+        <v>121</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60">
-        <f t="shared" si="1"/>
-        <v>6000</v>
+        <f t="shared" si="0"/>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61">
-        <f t="shared" si="1"/>
-        <v>6100</v>
+        <f t="shared" si="0"/>
+        <v>125</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62">
-        <f t="shared" si="1"/>
-        <v>6200</v>
+        <f t="shared" si="0"/>
+        <v>127</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63">
-        <f t="shared" si="1"/>
-        <v>6300</v>
+        <f t="shared" si="0"/>
+        <v>129</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64">
-        <f t="shared" si="1"/>
-        <v>6400</v>
+        <f t="shared" si="0"/>
+        <v>131</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65">
-        <f t="shared" si="1"/>
-        <v>6500</v>
+        <f t="shared" si="0"/>
+        <v>133</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66">
-        <f t="shared" si="1"/>
-        <v>6600</v>
+        <f t="shared" ref="A66:A100" si="1">ROW(A66) * 2 + 3</f>
+        <v>135</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67">
         <f t="shared" si="1"/>
-        <v>6700</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68">
         <f t="shared" si="1"/>
-        <v>6800</v>
+        <v>139</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69">
         <f t="shared" si="1"/>
-        <v>6900</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70">
         <f t="shared" si="1"/>
-        <v>7000</v>
+        <v>143</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71">
         <f t="shared" si="1"/>
-        <v>7100</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72">
-        <f t="shared" ref="A72:A100" si="2">ROW(A72) * 100</f>
-        <v>7200</v>
+        <f t="shared" si="1"/>
+        <v>147</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73">
-        <f t="shared" si="2"/>
-        <v>7300</v>
+        <f t="shared" si="1"/>
+        <v>149</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74">
-        <f t="shared" si="2"/>
-        <v>7400</v>
+        <f t="shared" si="1"/>
+        <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75">
-        <f t="shared" si="2"/>
-        <v>7500</v>
+        <f t="shared" si="1"/>
+        <v>153</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76">
-        <f t="shared" si="2"/>
-        <v>7600</v>
+        <f t="shared" si="1"/>
+        <v>155</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77">
-        <f t="shared" si="2"/>
-        <v>7700</v>
+        <f t="shared" si="1"/>
+        <v>157</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78">
-        <f t="shared" si="2"/>
-        <v>7800</v>
+        <f t="shared" si="1"/>
+        <v>159</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79">
-        <f t="shared" si="2"/>
-        <v>7900</v>
+        <f t="shared" si="1"/>
+        <v>161</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80">
-        <f t="shared" si="2"/>
-        <v>8000</v>
+        <f t="shared" si="1"/>
+        <v>163</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A81">
-        <f t="shared" si="2"/>
-        <v>8100</v>
+        <f t="shared" si="1"/>
+        <v>165</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A82">
-        <f t="shared" si="2"/>
-        <v>8200</v>
+        <f t="shared" si="1"/>
+        <v>167</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A83">
-        <f t="shared" si="2"/>
-        <v>8300</v>
+        <f t="shared" si="1"/>
+        <v>169</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A84">
-        <f t="shared" si="2"/>
-        <v>8400</v>
+        <f t="shared" si="1"/>
+        <v>171</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A85">
-        <f t="shared" si="2"/>
-        <v>8500</v>
+        <f t="shared" si="1"/>
+        <v>173</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A86">
-        <f t="shared" si="2"/>
-        <v>8600</v>
+        <f t="shared" si="1"/>
+        <v>175</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A87">
-        <f t="shared" si="2"/>
-        <v>8700</v>
+        <f t="shared" si="1"/>
+        <v>177</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A88">
-        <f t="shared" si="2"/>
-        <v>8800</v>
+        <f t="shared" si="1"/>
+        <v>179</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A89">
-        <f t="shared" si="2"/>
-        <v>8900</v>
+        <f t="shared" si="1"/>
+        <v>181</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A90">
-        <f t="shared" si="2"/>
-        <v>9000</v>
+        <f t="shared" si="1"/>
+        <v>183</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A91">
-        <f t="shared" si="2"/>
-        <v>9100</v>
+        <f t="shared" si="1"/>
+        <v>185</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A92">
-        <f t="shared" si="2"/>
-        <v>9200</v>
+        <f t="shared" si="1"/>
+        <v>187</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A93">
-        <f t="shared" si="2"/>
-        <v>9300</v>
+        <f t="shared" si="1"/>
+        <v>189</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A94">
-        <f t="shared" si="2"/>
-        <v>9400</v>
+        <f t="shared" si="1"/>
+        <v>191</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A95">
-        <f t="shared" si="2"/>
-        <v>9500</v>
+        <f t="shared" si="1"/>
+        <v>193</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A96">
-        <f t="shared" si="2"/>
-        <v>9600</v>
+        <f t="shared" si="1"/>
+        <v>195</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97">
-        <f t="shared" si="2"/>
-        <v>9700</v>
+        <f t="shared" si="1"/>
+        <v>197</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98">
-        <f t="shared" si="2"/>
-        <v>9800</v>
+        <f t="shared" si="1"/>
+        <v>199</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99">
-        <f t="shared" si="2"/>
-        <v>9900</v>
+        <f t="shared" si="1"/>
+        <v>201</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100">
-        <f t="shared" si="2"/>
-        <v>10000</v>
+        <f t="shared" si="1"/>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>